<commit_message>
feat: Introduce Snapsheet configuration and validation improvements
- Added SnapsheetConfig struct to manage configuration from a TOML file.
- Enhanced validation for address blocks and registers, including checks for duplicates and overlaps.
- Updated parse_component and parse_blocks functions to utilize configuration settings.
- Introduced collect_validation function to aggregate validation issues.
- Updated tests to cover new configuration and validation logic.
- Added example workbooks and scripts for easier testing and demonstration.
- Updated documentation to reflect changes in validation rules and configuration structure.
</commit_message>
<xml_diff>
--- a/example.xlsx
+++ b/example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/beribeli/Workarea/irgen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDDC6A2C-06DB-BC44-864A-2FEB24C3347E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA98CC92-D634-614C-8090-C66DDF59DAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="version" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="61">
   <si>
     <t>VENDOR</t>
   </si>
@@ -198,6 +198,18 @@
   </si>
   <si>
     <t>regb{n}, n=range(0, 2, 8)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x200</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>[63:0]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>rege{n}, n=range(0, 2, 8)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -257,10 +269,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -598,10 +610,10 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -622,8 +634,8 @@
       <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
       <c r="C4" s="1" t="s">
         <v>35</v>
       </c>
@@ -642,8 +654,8 @@
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
       <c r="C5" s="1" t="s">
         <v>37</v>
       </c>
@@ -662,8 +674,8 @@
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
       <c r="C6" s="1" t="s">
         <v>25</v>
       </c>
@@ -754,10 +766,10 @@
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -778,8 +790,8 @@
       <c r="H10" s="1"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
       <c r="C11" s="1" t="s">
         <v>25</v>
       </c>
@@ -817,7 +829,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="7.1640625" style="1" customWidth="1"/>
@@ -879,10 +891,10 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -902,8 +914,8 @@
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
       <c r="C4" s="1" t="s">
         <v>35</v>
       </c>
@@ -921,8 +933,8 @@
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
       <c r="C5" s="1" t="s">
         <v>37</v>
       </c>
@@ -940,8 +952,8 @@
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
       <c r="C6" s="1" t="s">
         <v>25</v>
       </c>
@@ -1028,7 +1040,7 @@
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>48</v>
       </c>
       <c r="B10" s="5" t="s">
@@ -1051,8 +1063,8 @@
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
       <c r="C11" s="1" t="s">
         <v>25</v>
       </c>
@@ -1070,10 +1082,10 @@
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>53</v>
       </c>
       <c r="C12" s="1" t="s">
@@ -1093,8 +1105,8 @@
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
       <c r="C13" s="1" t="s">
         <v>25</v>
       </c>
@@ -1115,7 +1127,7 @@
       <c r="A14" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -1128,6 +1140,26 @@
         <v>27</v>
       </c>
       <c r="G14" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E15" s="1">
+        <v>64</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>